<commit_message>
Refresh File1 workbook after V_overflow labels
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Retention_1200_File1_Composite.xlsx
+++ b/engineering/drainage-design/retention_volume/Retention_1200_File1_Composite.xlsx
@@ -6940,7 +6940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -7010,60 +7010,84 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • WSEmax = niveau max retenu a l'entree du Ø1200</t>
+          <t xml:space="preserve">  • V_hold (B31) = volume a RETENIR a l'entree du Ø1200 (m3)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Q_down max = pointe aval = pipe + overflow</t>
+          <t xml:space="preserve">  • V_overflow (B33) = volume qui a DEBORDE par la fosse (m3) = Σ Q_overflow×dt</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Split Q_1200 / Q_overflow a cette pointe</t>
+          <t xml:space="preserve">  • WSEmax = niveau max retenu a l'entree du Ø1200</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Q_down max = pointe aval = pipe + overflow</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Fichiers suivants (separes, pas encore dans ce classeur):</t>
+          <t xml:space="preserve">  • Split Q_1200 / Q_overflow a cette pointe</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  File 2 = comparaison pipe-only vs composite</t>
-        </is>
-      </c>
+      <c r="A17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  File 3 = series temporelles detaillees (Idee 4)</t>
+          <t>Important: V_hold ≠ V_overflow. V_hold = a stocker; V_overflow = parti a l'aval via fosse.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  File 4 = sensibilite crest (Idee 5)</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Fichiers suivants (separes, pas encore dans ce classeur):</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  File 2 = comparaison pipe-only vs composite</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  File 3 = series temporelles detaillees (Idee 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  File 4 = sensibilite crest (Idee 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Regenerer: python3 build_retention_file1_composite.py</t>
         </is>

</xml_diff>